<commit_message>
Actualizar archivos corregidos de documentación
</commit_message>
<xml_diff>
--- a/docs/Blacklog inicial.xlsx
+++ b/docs/Blacklog inicial.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrie\OneDrive\Escritorio\Semestre 3\Programacion Orientada a Objetos\Proyecto tetris\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrie\OneDrive\Escritorio\Semestre 3\Programacion Orientada a Objetos\Proyecto tetris\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2189EB7C-2C17-A640-979B-741EAB6172BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCEE1B27-CB53-4B43-9D00-CA286257EC94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{9529548D-A73A-425D-A87A-1FD54AAFD713}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="55">
   <si>
     <t>ID</t>
   </si>
@@ -77,83 +77,200 @@
     <t>HU7</t>
   </si>
   <si>
-    <t>Las piezas caen en una cuadrícula ubicada al centro. El jugador puede moverlas y rotarlas. Las líneas completas se eliminan correctamente y suman puntos.</t>
-  </si>
-  <si>
-    <t>Se muestra una vista previa clara de la siguiente pieza debajo de la cuadrícula. Se actualiza conforme avanza el juego.</t>
-  </si>
-  <si>
-    <t>La velocidad de caída aumenta por nivel. Las operaciones matemáticas al final de cada nivel se vuelven más complejas (más dígitos y operaciones).</t>
-  </si>
-  <si>
-    <t>Al completar un nivel, se presenta una operación matemática. Si la respuesta es correcta, avanza; si no, el juego reinicia desde el nivel 0 y el puntaje se reinicia.</t>
-  </si>
-  <si>
     <t>HU8</t>
   </si>
   <si>
     <t>HU9</t>
   </si>
   <si>
-    <t>Como jugador, quiero que las piezas del Tetris caigan y se acomoden correctamente en una cuadrícula central, para formar líneas y ganar puntos.</t>
-  </si>
-  <si>
-    <t>Como jugador, quiero que durante la partida se muestre el nivel actual en la parte superior izquierda y mi puntaje en la parte superior derecha, para seguir mi progreso.</t>
-  </si>
-  <si>
-    <t>Como jugador, quiero que en la parte inferior del área de juego aparezca la siguiente pieza que va a caer, para planificar mis movimientos.</t>
-  </si>
-  <si>
-    <t>Como jugador, quiero que el juego tenga 10 niveles con dificultad progresiva, para mantener el desafío conforme avanzo.</t>
-  </si>
-  <si>
-    <t>Como jugador, quiero resolver una operación matemática al terminar cada nivel, para avanzar al siguiente.</t>
-  </si>
-  <si>
-    <t>Como jugador, quiero que el juego termine si lleno una columna vertical, para mantener la mecánica clásica del Tetris.</t>
-  </si>
-  <si>
-    <t>Como jugador, quiero que mis puntajes se guarden localmente, para poder intentar superarlos después.</t>
-  </si>
-  <si>
-    <t>Como jugador, quiero que el juego tenga colores atractivos, para hacerlo más divertido y mantener la atención.</t>
-  </si>
-  <si>
-    <t>Los puntajes se guardan en un archivo local (TXT). Al iniciar el juego, se muestra el puntaje más alto alcanzado.</t>
+    <t>- Python está instalado. - La librería Pygame está instalada y operativa. - Se crea la estructura de carpetas del proyecto. - Se inicializa una ventana de juego básica.</t>
+  </si>
+  <si>
+    <t>Como jugador, quiero que las piezas de Tetris caigan desde la parte superior de la pantalla para poder interactuar con ellas.</t>
+  </si>
+  <si>
+    <t>- Se genera una pieza aleatoria en la parte superior central del tablero. - La pieza desciende a una velocidad constante (velocidad del Nivel 1).</t>
+  </si>
+  <si>
+    <t>Como jugador, quiero poder mover las piezas hacia la izquierda y la derecha para poder posicionarlas.</t>
+  </si>
+  <si>
+    <t>- Al presionar la tecla de flecha izquierda, la pieza se mueve una columna a la izquierda. - Al presionar la tecla de flecha derecha, la pieza se mueve una columna a la derecha. - La pieza no puede salirse de los límites laterales del área de juego.</t>
+  </si>
+  <si>
+    <t>Como jugador, quiero poder rotar las piezas para que encajen mejor en los espacios disponibles.</t>
+  </si>
+  <si>
+    <t>- Al presionar una tecla designada (ej. flecha arriba), la pieza activa rota 90 grados en sentido horario. - La rotación no permite que la pieza atraviese otras piezas ya colocadas o los límites del tablero.</t>
+  </si>
+  <si>
+    <t>Como jugador, quiero que las líneas horizontales completas desaparezcan y me den puntos, para sentir que progreso en el juego.</t>
+  </si>
+  <si>
+    <t>- Cuando una fila se llena por completo, se elimina del tablero. - Las filas superiores caen para ocupar el espacio vacío. - El puntaje del jugador aumenta por cada línea eliminada.</t>
+  </si>
+  <si>
+    <t>- Si una pieza se bloquea y una parte de ella queda fuera del límite superior del área de juego, la partida finaliza. - Se muestra una pantalla o mensaje de "Game Over".</t>
+  </si>
+  <si>
+    <t>- Después de eliminar un número determinado de líneas, el juego se pausa. - Aparece en pantalla una interfaz para resolver una operación matemática.</t>
   </si>
   <si>
     <r>
-      <t>Como jugador, quiero ver una pantalla de inicio simple con la opción "Jugar"</t>
+      <t xml:space="preserve">Como jugador del </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1B1C1D"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Nivel 1</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
+        <color rgb="FF1B1C1D"/>
+        <rFont val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> y el puntaje máximo alcanzado, para comenzar una partida fácilmente.</t>
+      <t>, quiero resolver sumas o restas de 1 dígito para poder pasar al siguiente nivel.</t>
     </r>
   </si>
   <si>
-    <t>La pantalla inicial muestra los botones "Jugar" e "Instrucciones". Al presionar "Jugar", inicia la partida.</t>
-  </si>
-  <si>
-    <t>Se visualiza el nivel actual en la parte superior central, así como el score en tiempo real.</t>
-  </si>
-  <si>
-    <t>El juego detecta cuando una columna se llena por completo y muestra un mensaje de “¡¡CASI!! Intenta otra vez” con opción para reiniciar.</t>
-  </si>
-  <si>
-    <t>La interfaz usa colores vivos al eliminar líneas o perder.</t>
+    <t>- Al final del Nivel 1, la operación generada es una suma o resta. - Los operandos son números de un solo dígito (0-9). - El jugador puede introducir su respuesta.</t>
+  </si>
+  <si>
+    <t>- Si la respuesta introducida es incorrecta, el estado del juego vuelve al inicio del Nivel 1. - El puntaje del jugador se restablece a 0.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Como jugador del </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1B1C1D"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Nivel 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1B1C1D"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, quiero resolver sumas o restas de 2 dígitos.</t>
+    </r>
+  </si>
+  <si>
+    <t>- Al final del Nivel 2, la operación generada es una suma o resta. - Los operandos son números de dos dígitos (10-99).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Como jugador del </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1B1C1D"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Nivel 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1B1C1D"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, quiero resolver multiplicaciones de 1 dígito.</t>
+    </r>
+  </si>
+  <si>
+    <t>- Al final del Nivel 3, la operación generada es una multiplicación. - Los operandos son números de un solo dígito.</t>
+  </si>
+  <si>
+    <t>- La velocidad de caída en el Nivel 2 es notablemente más rápida que en el Nivel 1. - La velocidad de caída en el Nivel 3 es la máxima del juego.</t>
+  </si>
+  <si>
+    <t>Como jugador, quiero ver en pantalla mi puntaje actual y el nivel en el que me encuentro.</t>
+  </si>
+  <si>
+    <t>- Un área de la interfaz de usuario muestra el puntaje en tiempo real. - Otro indicador muestra el nivel actual (1, 2 o 3).</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>- Al finalizar una partida, si el puntaje actual supera al récord guardado, este se actualiza. - El puntaje más alto se almacena en un archivo local para que persista entre sesiones de juego.</t>
+  </si>
+  <si>
+    <t>Como jugador, quiero una pantalla de inicio que muestre el título del juego, el puntaje más alto y un botón para "Iniciar Juego".</t>
+  </si>
+  <si>
+    <t>- Al ejecutar la aplicación, aparece una pantalla de bienvenida. - La pantalla muestra el récord de puntuación guardado. - Hay un botón o una instrucción de tecla para comenzar una nueva partida.</t>
+  </si>
+  <si>
+    <t>- Se utiliza una paleta de colores atractiva para el público infantil. - Las fuentes de texto son grandes y legibles. - El diseño general es simple e intuitivo.</t>
+  </si>
+  <si>
+    <t>Como desarrollador, necesito configurar el entorno de desarrollo con Python y la librería Pygame para poder iniciar la construcción del juego.</t>
+  </si>
+  <si>
+    <t>Como jugador, necesito que el juego termine si las piezas se apilan hasta la parte superior de la pantalla, como en el Tetris original.</t>
+  </si>
+  <si>
+    <t>Como jugador, al completar un nivel, quiero que se me presente una operación matemática para poder avanzar.</t>
+  </si>
+  <si>
+    <t>Como jugador, si mi respuesta a la operación es incorrecta, quiero que el juego y mi puntaje se reinicien para intentarlo de nuevo.</t>
+  </si>
+  <si>
+    <t>Como jugador, quiero que la velocidad de caída de las piezas aumente en cada nivel para que el juego sea más desafiante.</t>
+  </si>
+  <si>
+    <t>Como jugador, quiero que mi puntaje más alto se guarde para poder competir contra mí mismo en futuras partidas.</t>
+  </si>
+  <si>
+    <t>Como niño, quiero que el juego tenga una interfaz amigable, con colores vivos y elementos visuales claros para que sea más divertido y fácil de entender.</t>
+  </si>
+  <si>
+    <t>HU10</t>
+  </si>
+  <si>
+    <t>HU11</t>
+  </si>
+  <si>
+    <t>HU12</t>
+  </si>
+  <si>
+    <t>HU13</t>
+  </si>
+  <si>
+    <t>HU14</t>
+  </si>
+  <si>
+    <t>HU15</t>
+  </si>
+  <si>
+    <t>HU16</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,12 +279,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF1B1C1D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <color rgb="FF1B1C1D"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -178,7 +300,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -186,23 +308,119 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -538,159 +756,252 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF6848FF-A75F-479A-B46D-D30A0615EB70}">
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="10.76171875" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="C1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.97265625" customWidth="1"/>
-    <col min="2" max="2" width="41.56640625" customWidth="1"/>
-    <col min="4" max="4" width="48.96484375" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="41.5703125" customWidth="1"/>
+    <col min="4" max="4" width="49" customWidth="1"/>
+    <col min="6" max="6" width="57.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="3:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="3:6" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="D2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="3:6" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="3:6" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="3:6" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" ht="44.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="3:6" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="4" t="s">
+    </row>
+    <row r="11" spans="3:6" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="E11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="4" t="s">
+    <row r="12" spans="3:6" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="E12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+    <row r="13" spans="3:6" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="3:6" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="3:6" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="3:6" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="3:6" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>